<commit_message>
BD web: actualizar base sellin (BD_SELL_IN_NUVA.xlsx)
</commit_message>
<xml_diff>
--- a/1 venta sell in/BD_SELL_IN_NUVA.xlsx
+++ b/1 venta sell in/BD_SELL_IN_NUVA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conchaytoro365-my.sharepoint.com/personal/jose_vidal_conchaytoro_cl/Documents/Escritorio/Proyecto-Nuva-Oxi/1 venta sell in/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conchaytoro365-my.sharepoint.com/personal/jose_vidal_conchaytoro_cl/Documents/Escritorio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="14_{2093FD1B-1272-4C46-A2D8-8D2742D38FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F01B80E7-858A-494A-B9AA-0D4ABF489BE5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B98CD5A-773B-4EBE-A0B8-89E5CDB14841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{A457DA66-1803-4DEC-82CE-ADDD8E755DA3}"/>
+    <workbookView xWindow="28680" yWindow="2175" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{A457DA66-1803-4DEC-82CE-ADDD8E755DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="ANALISIS" sheetId="6" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <definedName name="DatosExternos_1" localSheetId="2">ref_SKU!$A$1:$F$7</definedName>
     <definedName name="DatosExternos_1" localSheetId="4">VENTAS!$A$1:$L$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -975,7 +975,7 @@
       </c>
       <c r="B3" s="5">
         <f>SUM(VENTAS!F:F)</f>
-        <v>92</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="L2">
         <f ca="1">IF(K2="",TODAY()-C2,K2-C2)</f>
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M2" t="s">
         <v>81</v>
@@ -1650,7 +1650,7 @@
         <v>14</v>
       </c>
       <c r="F2">
-        <v>12</v>
+        <v>1000</v>
       </c>
       <c r="G2">
         <v>19160</v>

</xml_diff>